<commit_message>
feat: SP/PC upload UI split + auto image processing (square crop, 600x600, JPEG, ≤2MB)
</commit_message>
<xml_diff>
--- a/CSV不足項目チェックシート.xlsx
+++ b/CSV不足項目チェックシート.xlsx
@@ -581,46 +581,46 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="n">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Step1</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>申請者情報</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>別名 姓の苗字チェック</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>CSV: 別名の姓にも苗字辞書チェックを適用</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>❌ 未該当 — 現フォームはsurnameのみ。aliasSurnameには苗字チェック未実装</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>✅ 実装済み — 現フォームはsurnameのみ。aliasSurnameには苗字チェック実装完了（attachSurnameAlert関数で全姓フィールドに適用）</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>別名「はい」→aliasSurnameに「SUZKI」入力→blur</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>苗字アラートが表示される</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="I3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>実装追加が必要なら対応可能</t>
         </is>
@@ -1273,134 +1273,134 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Step3</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>緊急連絡先</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>姓の苗字チェック</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>CSV: 候補にない場合はアラート表示</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>❌ 未該当 — 緊急連絡先の姓に苗字チェック未実装</t>
-        </is>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>✅ 実装済み — 緊急連絡先の姓に苗字チェック実装完了（attachSurnameAlert関数で全姓フィールドに適用）</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>緊急連絡先「はい」→姓に「SUZKI」入力→blur</t>
         </is>
       </c>
-      <c r="H19" s="5" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>苗字アラートが表示される</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr"/>
-      <c r="J19" s="5" t="inlineStr">
+      <c r="I19" s="7" t="inlineStr"/>
+      <c r="J19" s="7" t="inlineStr">
         <is>
           <t>実装追加が必要</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n">
+      <c r="A20" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Step3</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>緊急連絡先</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>電話番号 13文字制限</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="7" t="inlineStr">
         <is>
           <t>CSV: 文字数13文字以内</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>⚠️ 差異あり — 現テストは20文字</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="7" t="inlineStr">
         <is>
           <t>緊急連絡先電話番号に14桁入力</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H20" s="7" t="inlineStr">
         <is>
           <t>13文字で切り捨てられる</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr"/>
+      <c r="J20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="A21" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Step3</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>両親情報</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>父/母 姓の苗字チェック</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>CSV: 候補にない場合はアラート表示</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>❌ 未該当 — 両親の姓に苗字チェック未実装</t>
-        </is>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>✅ 実装済み — 両親の姓に苗字チェック実装完了（attachSurnameAlert関数で全姓フィールドに適用）</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>父の姓に「TNAKA」入力→blur</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>苗字アラートが表示される</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr">
+      <c r="I21" s="7" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr">
         <is>
           <t>実装追加が必要</t>
         </is>

</xml_diff>